<commit_message>
Verze 0.21.1: Ceník prací – doplněny všechny položky ze starších verzí, žádná se neztratí, kódy bez kolizí
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VRp7EPrDBAjXFErf59Agpz
</commit_message>
<xml_diff>
--- a/data/cenik-praci-2026.xlsx
+++ b/data/cenik-praci-2026.xlsx
@@ -64,7 +64,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +81,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -94,10 +99,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7554,6 +7560,726 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-016</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Aplikace tekuté hydroizolace (1. vrstva)</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>Nátěr tekutou hydroizolací válečkem / štětcem v 1. vrstvě na penetrovaný podklad</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-017</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Aplikace tekuté hydroizolace (2. vrstva křížově)</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>Druhá vrstva tekuté hydroizolace nanesená křížově přes 1. vrstvu po zaschnutí</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-018</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Aplikace 2K reaktivní hydroizolační stěrky (exteriér/balkón)</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>Dvousložková reaktivní hydroizolační stěrka pro exteriér a balkóny, nanášená ve 2 vrstvách</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-019</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Lepení hydroizolační těsnicí pásky do koutů a rohů</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>Vlepování hydroizolační těsnicí pásky do koutů a rohů do čerstvé hydroizolace</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H206" s="3" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-020</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Montáž hydroizolačních vnitřních / vnějších rohů</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>Osazení hydroizolačních vnitřních / vnějších rohů do čerstvé hydroizolace</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-021</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Montáž pružné hydroizolační manžety pro vodovodní vývod</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>Osazení pružné manžety na vodovodní vývod a zatření hydroizolací</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H208" s="3" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-022</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Montáž těsnicí manžety pod podlahový sprchový žlab</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>Osazení těsnicí manžety pod podlahový sprchový žlab a zatření hydroizolací</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-023</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Montáž separační / odvlhčovací / roznášecí rohože pod dlažbu</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>Pokládka separační / odvlhčovací / roznášecí rohože pod dlažbu</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-024</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Montáž sprchového nerezového žlabu vč. usazení a napojení</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>Usazení nerezového sprchového žlabu do spádu a napojení na odpad</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-025</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Tlaková zkouška těsnosti hydroizolace (přetlakové zatopení)</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>soubor</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F212" s="3" t="inlineStr">
+        <is>
+          <t>Přetlaková zkouška těsnosti hydroizolace zatopením, kontrola po stanovenou dobu</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-026</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Napojení hydroizolace na podlahovou vpusť / odtok (manžeta)</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>Napojení hydroizolace na podlahovou vpusť / odtok pomocí manžety</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>4. Hydroizolace a těsnění</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>HYDR-027</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Montáž okrajového dilatačního pásku a akustické izolace pod dlažbu</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>Montáž okrajového dilatačního pásku a akustické izolace po obvodu pod dlažbu</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>6. Kamenické opracování a detaily</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>KAM-004</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Vrtání otvoru do gresu / přírodního kamene do průměru 35 mm</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>Diamantové vrtání otvoru korunkou do průměru 35 mm</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>6. Kamenické opracování a detaily</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>KAM-005</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Vrtání velkého otvoru do gresu (ZTI, odpady 50–110 mm)</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>Diamantové vrtání velkého otvoru (50–110 mm) pro ZTI a odpady</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>6. Kamenické opracování a detaily</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>KAM-006</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Výřez otvoru pro elektrokrabice / zásuvky</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>Vyříznutí otvoru pro elektrokrabici / zásuvku v obkladu</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>3. Zednické práce a vyrovnání</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>NIV-008</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>Broušení / frézování podkladu diamantovou bruskou</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>Odstranění lepidla a mléka</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>10. Finální čištění, úklid a předání díla</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>UKL-009</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Přípravný úklid staveniště před zahájením prací (vysátí prachu, odmetení, hrubé očištění podkladu)</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>Vysátí průmyslovým vysavačem a očištění zdiva/podlahy před penetrací</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>10. Finální čištění, úklid a předání díla</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>UKL-010</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>Průběžný úklid během realizace (vynášení suti v pytlích, úklid odpadu z lepení a sádrokartonů)</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>Denní průběžné udržování čistoty a třídění odpadu na staveništi</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>10. Finální čištění, úklid a předání díla</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>UKL-011</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Finální generální úklid po dokončení prací (odstranění cementových povlaků, zaleštění, mytí)</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>Hloubkové mytí obkladů, dlažeb, zařizovacích předmětů a stržení ochranných fólií</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>10. Finální čištění, úklid a předání díla</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>UKL-012</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>Strojní / chemické odstraňování epoxidového závoje a zbytkového tmelu</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>Použití speciálních chemických čističů epoxidových spár vč. zaleštění gresu</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7566,7 +8292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8495,6 +9221,42 @@
           <t>Nově zařazeno 2026</t>
         </is>
       </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Výrobky</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>PRD-054</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Výroba lepeného květináče / truhlíku z gresové dlažby</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Včetně vnitřní hydroizolace</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H26"/>
@@ -9587,7 +10349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9852,6 +10614,42 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Schody</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SCH-007</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Obložení schodišťového stupně (nášlap + podstupnice)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>680</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Obložení rovných schodů</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9864,7 +10662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10373,6 +11171,186 @@
           <t>Nově zařazeno 2026</t>
         </is>
       </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>1. Pokládka a mozaika</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>BAZ-014</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Lepení mozaiky v bazénu / parní sauně na epoxidový tmel</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>950</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Lepení skleněné / keramické mozaiky s dodržením spárořezu</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>1. Pokládka a mozaika</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>BAZ-015</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Pokládka mozaiky na zakřivených plochách bazénových lavic a lehátek</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Anatomicky tvarované sedáky, lelehátka a masážní bazénové prvky</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>1. Pokládka a mozaika</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>BAZ-016</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Obložení přepadové hrany / bazénové drážky protiskluzovými tvarovkami</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Osazení speciálních přepadových hran (St. Moritz, Wiesbaden)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>1. Pokládka a mozaika</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>BAZ-017</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Lepení protiskluzové dlažby R11 / R12 na schodech a okolo bazénu</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Pokládka bezpečnostní dlažby vč. nerezových / keramických nosů</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2. Bazénová chemie a hydroizolace</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>BAZ-018</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Aplikace chemicky odolné dvousložkové cementové hydroizolace (přetlak / podtlak)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>380</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Odolnost vůči chlóru, slané vodě a agresivní chemii</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H14"/>
@@ -12057,7 +13035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13352,6 +14330,42 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Standardní obklady</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>OBK-001</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Lepení obkladu standardního formátu (20x20 až 30x60 cm)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>550</v>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Standardní lepení na tmel C2TE</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13364,7 +14378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -14973,6 +15987,42 @@
           <t>Nově zařazeno 2026</t>
         </is>
       </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Standardní dlažba</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>DLZ-001</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Pokládka dlažby standardního formátu (30x30 až 60x60 cm)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Lepení na tmel C2TE S1</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Zachováno ze starší verze</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H51"/>

</xml_diff>

<commit_message>
Verze 0.23.0: Průvodce – lepidla podle formátu, Kerapoxy Easy Design + čistič, Mapelastic Smart + Mapenet, ředění Primeru G, volba separace a silikonu
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VRp7EPrDBAjXFErf59Agpz
</commit_message>
<xml_diff>
--- a/data/cenik-praci-2026.xlsx
+++ b/data/cenik-praci-2026.xlsx
@@ -1203,7 +1203,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broušení, očištění a odmaštění podkladu</t>
+          <t>Broušení podkladu vč. ořezu dilatačního pásu po betonáži a očištění</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Broušení podkladu, odsátí prachu a odmaštění pro dobrou přilnavost lepidla</t>
+          <t>Broušení brusnou, ořez přečnívajícího dilatačního pásu po betonáži, očištění; bez odmaštění (beton, anhydrit)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>